<commit_message>
v-A: bare gang search mixes boxes, mud rings and plates; DV34 unlocked on the assembly-hours sheet
"1 gang", "2 gang", "3 gang" (and "double gang") showed only wall plates in
the top five. rankMaterialHits now takes turns box -> mud ring -> plate for a
query that is a gang count and nothing else; a row naming a different count
goes last. "2 gang box/plate/mud ring" rank exactly as before. 7 new guards
in server/materialSearchRank.test.ts are red on the old code.

pricing/assembly-hours-starter.xlsx rebuilt ONLY (--only assembly-hours,
15 NEW marks kept): DV34 loads since 7641bb1, so its row is no longer grey,
noted or input-locked, and the loader accepts its hours (dry run checked).
Pricing and labor sheets untouched.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pricing/assembly-hours-starter.xlsx
+++ b/pricing/assembly-hours-starter.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="463">
-  <si>
-    <t>STARTER ASSEMBLY HOURS — every starter (183, 1 HELD, 15 NEW since the last version — filter the 'New' column). Your top-30 commercial list first, then the top-30 residential, then the rest. Type YELLOW 'MY HOURS' per assembly (one installed). 'Hours now' is what ships today (blank = not set). Leave blank to keep it. Grey = HELD, leave blank. Send the file back to Track A — do NOT edit hours in the app for this.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="462">
+  <si>
+    <t>STARTER ASSEMBLY HOURS — every starter (183, 15 NEW since the last version — filter the 'New' column). Your top-30 commercial list first, then the top-30 residential, then the rest. Type YELLOW 'MY HOURS' per assembly (one installed). 'Hours now' is what ships today (blank = not set). Leave blank to keep it. Grey = HELD, leave blank. Send the file back to Track A — do NOT edit hours in the app for this.</t>
   </si>
   <si>
     <t>#</t>
@@ -824,9 +824,6 @@
     <t>Surface raceway receptacle (block wall)</t>
   </si>
   <si>
-    <t>HELD - no 700 plate yet. Not seeded until the catalog has: Surface raceway device plate, 700 series. Leave MY HOURS blank.</t>
-  </si>
-  <si>
     <t>NEW</t>
   </si>
   <si>
@@ -1388,7 +1385,7 @@
     <t>HELD</t>
   </si>
   <si>
-    <t>DV34 Surface raceway receptacle (block wall) — grey, and refuses input. It is listed so the sheet is complete, but it is not seeded yet; leave it blank. See its Notes.</t>
+    <t>None.</t>
   </si>
   <si>
     <t>Not in this sheet</t>
@@ -1419,7 +1416,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1429,11 +1426,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2A8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -1454,15 +1446,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3840,7 +3831,7 @@
       </c>
       <c r="I95" s="3"/>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>94</v>
       </c>
@@ -3859,32 +3850,29 @@
       <c r="G96" t="s">
         <v>269</v>
       </c>
-      <c r="I96" s="4"/>
-      <c r="J96" s="2" t="s">
-        <v>270</v>
-      </c>
+      <c r="I96" s="3"/>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>95</v>
       </c>
-      <c r="B97" s="5" t="s">
+      <c r="B97" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="C97" t="s">
+        <v>201</v>
+      </c>
+      <c r="D97" t="s">
+        <v>12</v>
+      </c>
+      <c r="E97" t="s">
         <v>271</v>
-      </c>
-      <c r="C97" t="s">
-        <v>201</v>
-      </c>
-      <c r="D97" t="s">
-        <v>12</v>
-      </c>
-      <c r="E97" t="s">
-        <v>272</v>
       </c>
       <c r="F97" t="s">
         <v>18</v>
       </c>
       <c r="G97" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I97" s="3"/>
     </row>
@@ -3892,8 +3880,8 @@
       <c r="A98">
         <v>96</v>
       </c>
-      <c r="B98" s="5" t="s">
-        <v>271</v>
+      <c r="B98" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C98" t="s">
         <v>201</v>
@@ -3902,13 +3890,13 @@
         <v>138</v>
       </c>
       <c r="E98" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F98" t="s">
         <v>18</v>
       </c>
       <c r="G98" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I98" s="3"/>
     </row>
@@ -3916,8 +3904,8 @@
       <c r="A99">
         <v>97</v>
       </c>
-      <c r="B99" s="5" t="s">
-        <v>271</v>
+      <c r="B99" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C99" t="s">
         <v>201</v>
@@ -3926,13 +3914,13 @@
         <v>138</v>
       </c>
       <c r="E99" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F99" t="s">
         <v>18</v>
       </c>
       <c r="G99" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I99" s="3"/>
     </row>
@@ -3940,8 +3928,8 @@
       <c r="A100">
         <v>98</v>
       </c>
-      <c r="B100" s="5" t="s">
-        <v>271</v>
+      <c r="B100" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C100" t="s">
         <v>201</v>
@@ -3950,13 +3938,13 @@
         <v>138</v>
       </c>
       <c r="E100" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F100" t="s">
         <v>18</v>
       </c>
       <c r="G100" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="I100" s="3"/>
     </row>
@@ -3971,13 +3959,13 @@
         <v>12</v>
       </c>
       <c r="E101" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F101" t="s">
         <v>105</v>
       </c>
       <c r="G101" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I101" s="3"/>
     </row>
@@ -3992,13 +3980,13 @@
         <v>12</v>
       </c>
       <c r="E102" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F102" t="s">
         <v>105</v>
       </c>
       <c r="G102" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I102" s="3"/>
     </row>
@@ -4013,13 +4001,13 @@
         <v>12</v>
       </c>
       <c r="E103" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F103" t="s">
         <v>105</v>
       </c>
       <c r="G103" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I103" s="3"/>
     </row>
@@ -4034,13 +4022,13 @@
         <v>12</v>
       </c>
       <c r="E104" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F104" t="s">
         <v>105</v>
       </c>
       <c r="G104" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I104" s="3"/>
     </row>
@@ -4055,13 +4043,13 @@
         <v>138</v>
       </c>
       <c r="E105" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F105" t="s">
         <v>105</v>
       </c>
       <c r="G105" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I105" s="3"/>
     </row>
@@ -4076,13 +4064,13 @@
         <v>138</v>
       </c>
       <c r="E106" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F106" t="s">
         <v>105</v>
       </c>
       <c r="G106" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I106" s="3"/>
     </row>
@@ -4097,13 +4085,13 @@
         <v>138</v>
       </c>
       <c r="E107" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F107" t="s">
         <v>105</v>
       </c>
       <c r="G107" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I107" s="3"/>
     </row>
@@ -4118,13 +4106,13 @@
         <v>12</v>
       </c>
       <c r="E108" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F108" t="s">
         <v>105</v>
       </c>
       <c r="G108" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I108" s="3"/>
     </row>
@@ -4139,13 +4127,13 @@
         <v>12</v>
       </c>
       <c r="E109" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F109" t="s">
         <v>105</v>
       </c>
       <c r="G109" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I109" s="3"/>
     </row>
@@ -4160,13 +4148,13 @@
         <v>12</v>
       </c>
       <c r="E110" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F110" t="s">
         <v>105</v>
       </c>
       <c r="G110" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I110" s="3"/>
     </row>
@@ -4181,13 +4169,13 @@
         <v>12</v>
       </c>
       <c r="E111" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F111" t="s">
         <v>105</v>
       </c>
       <c r="G111" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I111" s="3"/>
     </row>
@@ -4202,13 +4190,13 @@
         <v>12</v>
       </c>
       <c r="E112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F112" t="s">
         <v>105</v>
       </c>
       <c r="G112" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I112" s="3"/>
     </row>
@@ -4223,13 +4211,13 @@
         <v>12</v>
       </c>
       <c r="E113" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F113" t="s">
         <v>105</v>
       </c>
       <c r="G113" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I113" s="3"/>
     </row>
@@ -4244,13 +4232,13 @@
         <v>12</v>
       </c>
       <c r="E114" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F114" t="s">
         <v>105</v>
       </c>
       <c r="G114" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I114" s="3"/>
     </row>
@@ -4265,13 +4253,13 @@
         <v>138</v>
       </c>
       <c r="E115" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F115" t="s">
         <v>105</v>
       </c>
       <c r="G115" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I115" s="3"/>
     </row>
@@ -4286,13 +4274,13 @@
         <v>53</v>
       </c>
       <c r="E116" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F116" t="s">
         <v>105</v>
       </c>
       <c r="G116" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I116" s="3"/>
     </row>
@@ -4307,13 +4295,13 @@
         <v>138</v>
       </c>
       <c r="E117" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F117" t="s">
         <v>105</v>
       </c>
       <c r="G117" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="I117" s="3"/>
     </row>
@@ -4328,13 +4316,13 @@
         <v>138</v>
       </c>
       <c r="E118" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F118" t="s">
         <v>105</v>
       </c>
       <c r="G118" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I118" s="3"/>
     </row>
@@ -4349,13 +4337,13 @@
         <v>138</v>
       </c>
       <c r="E119" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F119" t="s">
         <v>105</v>
       </c>
       <c r="G119" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I119" s="3"/>
     </row>
@@ -4370,13 +4358,13 @@
         <v>138</v>
       </c>
       <c r="E120" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F120" t="s">
         <v>105</v>
       </c>
       <c r="G120" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I120" s="3"/>
     </row>
@@ -4391,13 +4379,13 @@
         <v>138</v>
       </c>
       <c r="E121" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F121" t="s">
         <v>105</v>
       </c>
       <c r="G121" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I121" s="3"/>
     </row>
@@ -4412,13 +4400,13 @@
         <v>138</v>
       </c>
       <c r="E122" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F122" t="s">
         <v>105</v>
       </c>
       <c r="G122" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="I122" s="3"/>
     </row>
@@ -4433,13 +4421,13 @@
         <v>138</v>
       </c>
       <c r="E123" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F123" t="s">
         <v>105</v>
       </c>
       <c r="G123" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="I123" s="3"/>
     </row>
@@ -4454,13 +4442,13 @@
         <v>138</v>
       </c>
       <c r="E124" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F124" t="s">
         <v>105</v>
       </c>
       <c r="G124" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="I124" s="3"/>
     </row>
@@ -4475,13 +4463,13 @@
         <v>12</v>
       </c>
       <c r="E125" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F125" t="s">
         <v>41</v>
       </c>
       <c r="G125" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I125" s="3"/>
     </row>
@@ -4496,13 +4484,13 @@
         <v>53</v>
       </c>
       <c r="E126" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F126" t="s">
         <v>41</v>
       </c>
       <c r="G126" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I126" s="3"/>
     </row>
@@ -4517,13 +4505,13 @@
         <v>12</v>
       </c>
       <c r="E127" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F127" t="s">
         <v>41</v>
       </c>
       <c r="G127" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="I127" s="3"/>
     </row>
@@ -4538,13 +4526,13 @@
         <v>53</v>
       </c>
       <c r="E128" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F128" t="s">
         <v>41</v>
       </c>
       <c r="G128" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="I128" s="3"/>
     </row>
@@ -4559,13 +4547,13 @@
         <v>12</v>
       </c>
       <c r="E129" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F129" t="s">
         <v>41</v>
       </c>
       <c r="G129" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I129" s="3"/>
     </row>
@@ -4580,13 +4568,13 @@
         <v>138</v>
       </c>
       <c r="E130" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F130" t="s">
         <v>41</v>
       </c>
       <c r="G130" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="I130" s="3"/>
     </row>
@@ -4601,13 +4589,13 @@
         <v>53</v>
       </c>
       <c r="E131" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F131" t="s">
         <v>41</v>
       </c>
       <c r="G131" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="I131" s="3"/>
     </row>
@@ -4622,13 +4610,13 @@
         <v>53</v>
       </c>
       <c r="E132" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F132" t="s">
         <v>41</v>
       </c>
       <c r="G132" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="I132" s="3"/>
     </row>
@@ -4643,13 +4631,13 @@
         <v>12</v>
       </c>
       <c r="E133" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F133" t="s">
         <v>14</v>
       </c>
       <c r="G133" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="I133" s="3"/>
     </row>
@@ -4657,8 +4645,8 @@
       <c r="A134">
         <v>132</v>
       </c>
-      <c r="B134" s="5" t="s">
-        <v>271</v>
+      <c r="B134" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C134" t="s">
         <v>201</v>
@@ -4667,13 +4655,13 @@
         <v>12</v>
       </c>
       <c r="E134" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F134" t="s">
         <v>14</v>
       </c>
       <c r="G134" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="I134" s="3"/>
     </row>
@@ -4681,8 +4669,8 @@
       <c r="A135">
         <v>133</v>
       </c>
-      <c r="B135" s="5" t="s">
-        <v>271</v>
+      <c r="B135" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C135" t="s">
         <v>201</v>
@@ -4691,13 +4679,13 @@
         <v>12</v>
       </c>
       <c r="E135" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F135" t="s">
         <v>14</v>
       </c>
       <c r="G135" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="I135" s="3"/>
     </row>
@@ -4705,8 +4693,8 @@
       <c r="A136">
         <v>134</v>
       </c>
-      <c r="B136" s="5" t="s">
-        <v>271</v>
+      <c r="B136" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C136" t="s">
         <v>201</v>
@@ -4715,13 +4703,13 @@
         <v>12</v>
       </c>
       <c r="E136" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F136" t="s">
         <v>14</v>
       </c>
       <c r="G136" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="I136" s="3"/>
     </row>
@@ -4736,13 +4724,13 @@
         <v>138</v>
       </c>
       <c r="E137" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="F137" t="s">
         <v>14</v>
       </c>
       <c r="G137" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="I137" s="3"/>
     </row>
@@ -4757,13 +4745,13 @@
         <v>53</v>
       </c>
       <c r="E138" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F138" t="s">
         <v>14</v>
       </c>
       <c r="G138" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I138" s="3"/>
     </row>
@@ -4778,13 +4766,13 @@
         <v>53</v>
       </c>
       <c r="E139" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="F139" t="s">
         <v>14</v>
       </c>
       <c r="G139" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I139" s="3"/>
     </row>
@@ -4799,13 +4787,13 @@
         <v>53</v>
       </c>
       <c r="E140" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F140" t="s">
         <v>14</v>
       </c>
       <c r="G140" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I140" s="3"/>
     </row>
@@ -4820,13 +4808,13 @@
         <v>138</v>
       </c>
       <c r="E141" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F141" t="s">
         <v>14</v>
       </c>
       <c r="G141" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I141" s="3"/>
     </row>
@@ -4841,13 +4829,13 @@
         <v>138</v>
       </c>
       <c r="E142" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F142" t="s">
         <v>14</v>
       </c>
       <c r="G142" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I142" s="3"/>
     </row>
@@ -4862,13 +4850,13 @@
         <v>138</v>
       </c>
       <c r="E143" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F143" t="s">
         <v>14</v>
       </c>
       <c r="G143" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I143" s="3"/>
     </row>
@@ -4883,13 +4871,13 @@
         <v>138</v>
       </c>
       <c r="E144" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F144" t="s">
         <v>14</v>
       </c>
       <c r="G144" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="I144" s="3"/>
     </row>
@@ -4904,13 +4892,13 @@
         <v>53</v>
       </c>
       <c r="E145" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F145" t="s">
         <v>14</v>
       </c>
       <c r="G145" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="I145" s="3"/>
     </row>
@@ -4925,13 +4913,13 @@
         <v>138</v>
       </c>
       <c r="E146" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F146" t="s">
         <v>14</v>
       </c>
       <c r="G146" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="I146" s="3"/>
     </row>
@@ -4946,13 +4934,13 @@
         <v>138</v>
       </c>
       <c r="E147" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F147" t="s">
         <v>14</v>
       </c>
       <c r="G147" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="I147" s="3"/>
     </row>
@@ -4967,13 +4955,13 @@
         <v>12</v>
       </c>
       <c r="E148" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F148" t="s">
         <v>14</v>
       </c>
       <c r="G148" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="I148" s="3"/>
     </row>
@@ -4988,13 +4976,13 @@
         <v>12</v>
       </c>
       <c r="E149" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F149" t="s">
         <v>14</v>
       </c>
       <c r="G149" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="I149" s="3"/>
     </row>
@@ -5009,13 +4997,13 @@
         <v>12</v>
       </c>
       <c r="E150" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F150" t="s">
         <v>14</v>
       </c>
       <c r="G150" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="I150" s="3"/>
     </row>
@@ -5030,13 +5018,13 @@
         <v>12</v>
       </c>
       <c r="E151" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F151" t="s">
         <v>14</v>
       </c>
       <c r="G151" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I151" s="3"/>
     </row>
@@ -5051,13 +5039,13 @@
         <v>12</v>
       </c>
       <c r="E152" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F152" t="s">
         <v>14</v>
       </c>
       <c r="G152" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="I152" s="3"/>
     </row>
@@ -5065,8 +5053,8 @@
       <c r="A153">
         <v>151</v>
       </c>
-      <c r="B153" s="5" t="s">
-        <v>271</v>
+      <c r="B153" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C153" t="s">
         <v>201</v>
@@ -5075,13 +5063,13 @@
         <v>53</v>
       </c>
       <c r="E153" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F153" t="s">
         <v>14</v>
       </c>
       <c r="G153" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="I153" s="3"/>
     </row>
@@ -5089,8 +5077,8 @@
       <c r="A154">
         <v>152</v>
       </c>
-      <c r="B154" s="5" t="s">
-        <v>271</v>
+      <c r="B154" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C154" t="s">
         <v>201</v>
@@ -5099,13 +5087,13 @@
         <v>53</v>
       </c>
       <c r="E154" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F154" t="s">
         <v>14</v>
       </c>
       <c r="G154" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I154" s="3"/>
     </row>
@@ -5113,8 +5101,8 @@
       <c r="A155">
         <v>153</v>
       </c>
-      <c r="B155" s="5" t="s">
-        <v>271</v>
+      <c r="B155" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C155" t="s">
         <v>201</v>
@@ -5123,13 +5111,13 @@
         <v>53</v>
       </c>
       <c r="E155" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F155" t="s">
         <v>14</v>
       </c>
       <c r="G155" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I155" s="3"/>
     </row>
@@ -5144,13 +5132,13 @@
         <v>12</v>
       </c>
       <c r="E156" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F156" t="s">
         <v>89</v>
       </c>
       <c r="G156" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="I156" s="3"/>
     </row>
@@ -5165,13 +5153,13 @@
         <v>12</v>
       </c>
       <c r="E157" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F157" t="s">
         <v>89</v>
       </c>
       <c r="G157" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="I157" s="3"/>
     </row>
@@ -5186,13 +5174,13 @@
         <v>12</v>
       </c>
       <c r="E158" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F158" t="s">
         <v>89</v>
       </c>
       <c r="G158" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="I158" s="3"/>
     </row>
@@ -5207,13 +5195,13 @@
         <v>12</v>
       </c>
       <c r="E159" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F159" t="s">
         <v>89</v>
       </c>
       <c r="G159" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="I159" s="3"/>
     </row>
@@ -5228,13 +5216,13 @@
         <v>138</v>
       </c>
       <c r="E160" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F160" t="s">
         <v>89</v>
       </c>
       <c r="G160" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I160" s="3"/>
     </row>
@@ -5249,13 +5237,13 @@
         <v>138</v>
       </c>
       <c r="E161" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F161" t="s">
         <v>89</v>
       </c>
       <c r="G161" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I161" s="3"/>
     </row>
@@ -5270,13 +5258,13 @@
         <v>53</v>
       </c>
       <c r="E162" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F162" t="s">
         <v>89</v>
       </c>
       <c r="G162" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="I162" s="3"/>
     </row>
@@ -5291,13 +5279,13 @@
         <v>138</v>
       </c>
       <c r="E163" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F163" t="s">
         <v>89</v>
       </c>
       <c r="G163" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="I163" s="3"/>
     </row>
@@ -5312,13 +5300,13 @@
         <v>12</v>
       </c>
       <c r="E164" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F164" t="s">
         <v>89</v>
       </c>
       <c r="G164" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I164" s="3"/>
     </row>
@@ -5333,13 +5321,13 @@
         <v>138</v>
       </c>
       <c r="E165" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F165" t="s">
         <v>89</v>
       </c>
       <c r="G165" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I165" s="3"/>
     </row>
@@ -5354,13 +5342,13 @@
         <v>138</v>
       </c>
       <c r="E166" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F166" t="s">
         <v>89</v>
       </c>
       <c r="G166" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I166" s="3"/>
     </row>
@@ -5368,8 +5356,8 @@
       <c r="A167">
         <v>165</v>
       </c>
-      <c r="B167" s="5" t="s">
-        <v>271</v>
+      <c r="B167" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C167" t="s">
         <v>201</v>
@@ -5378,13 +5366,13 @@
         <v>12</v>
       </c>
       <c r="E167" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F167" t="s">
         <v>85</v>
       </c>
       <c r="G167" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="I167" s="3"/>
     </row>
@@ -5392,8 +5380,8 @@
       <c r="A168">
         <v>166</v>
       </c>
-      <c r="B168" s="5" t="s">
-        <v>271</v>
+      <c r="B168" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C168" t="s">
         <v>201</v>
@@ -5402,13 +5390,13 @@
         <v>138</v>
       </c>
       <c r="E168" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F168" t="s">
         <v>85</v>
       </c>
       <c r="G168" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I168" s="3"/>
     </row>
@@ -5416,8 +5404,8 @@
       <c r="A169">
         <v>167</v>
       </c>
-      <c r="B169" s="5" t="s">
-        <v>271</v>
+      <c r="B169" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C169" t="s">
         <v>201</v>
@@ -5426,13 +5414,13 @@
         <v>138</v>
       </c>
       <c r="E169" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F169" t="s">
         <v>85</v>
       </c>
       <c r="G169" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="I169" s="3"/>
     </row>
@@ -5440,8 +5428,8 @@
       <c r="A170">
         <v>168</v>
       </c>
-      <c r="B170" s="5" t="s">
-        <v>271</v>
+      <c r="B170" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C170" t="s">
         <v>201</v>
@@ -5450,13 +5438,13 @@
         <v>138</v>
       </c>
       <c r="E170" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="F170" t="s">
         <v>85</v>
       </c>
       <c r="G170" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="I170" s="3"/>
     </row>
@@ -5464,8 +5452,8 @@
       <c r="A171">
         <v>169</v>
       </c>
-      <c r="B171" s="5" t="s">
-        <v>271</v>
+      <c r="B171" s="4" t="s">
+        <v>270</v>
       </c>
       <c r="C171" t="s">
         <v>201</v>
@@ -5474,13 +5462,13 @@
         <v>138</v>
       </c>
       <c r="E171" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F171" t="s">
         <v>85</v>
       </c>
       <c r="G171" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I171" s="3"/>
     </row>
@@ -5495,13 +5483,13 @@
         <v>53</v>
       </c>
       <c r="E172" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="F172" t="s">
         <v>85</v>
       </c>
       <c r="G172" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H172">
         <v>8</v>
@@ -5519,13 +5507,13 @@
         <v>53</v>
       </c>
       <c r="E173" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F173" t="s">
         <v>85</v>
       </c>
       <c r="G173" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="I173" s="3"/>
     </row>
@@ -5540,13 +5528,13 @@
         <v>138</v>
       </c>
       <c r="E174" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F174" t="s">
         <v>85</v>
       </c>
       <c r="G174" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="I174" s="3"/>
     </row>
@@ -5561,13 +5549,13 @@
         <v>53</v>
       </c>
       <c r="E175" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F175" t="s">
         <v>85</v>
       </c>
       <c r="G175" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="I175" s="3"/>
     </row>
@@ -5582,13 +5570,13 @@
         <v>53</v>
       </c>
       <c r="E176" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="F176" t="s">
         <v>85</v>
       </c>
       <c r="G176" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I176" s="3"/>
     </row>
@@ -5603,13 +5591,13 @@
         <v>138</v>
       </c>
       <c r="E177" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="F177" t="s">
         <v>85</v>
       </c>
       <c r="G177" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I177" s="3"/>
     </row>
@@ -5624,13 +5612,13 @@
         <v>53</v>
       </c>
       <c r="E178" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="F178" t="s">
         <v>85</v>
       </c>
       <c r="G178" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="I178" s="3"/>
     </row>
@@ -5645,13 +5633,13 @@
         <v>12</v>
       </c>
       <c r="E179" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="F179" t="s">
         <v>85</v>
       </c>
       <c r="G179" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I179" s="3"/>
     </row>
@@ -5666,13 +5654,13 @@
         <v>12</v>
       </c>
       <c r="E180" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="F180" t="s">
         <v>85</v>
       </c>
       <c r="G180" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I180" s="3"/>
     </row>
@@ -5687,13 +5675,13 @@
         <v>12</v>
       </c>
       <c r="E181" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="F181" t="s">
         <v>85</v>
       </c>
       <c r="G181" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="I181" s="3"/>
     </row>
@@ -5708,13 +5696,13 @@
         <v>12</v>
       </c>
       <c r="E182" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F182" t="s">
         <v>85</v>
       </c>
       <c r="G182" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="I182" s="3"/>
     </row>
@@ -5729,13 +5717,13 @@
         <v>53</v>
       </c>
       <c r="E183" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F183" t="s">
         <v>85</v>
       </c>
       <c r="G183" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="I183" s="3"/>
     </row>
@@ -5750,13 +5738,13 @@
         <v>12</v>
       </c>
       <c r="E184" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F184" t="s">
         <v>85</v>
       </c>
       <c r="G184" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="I184" s="3"/>
     </row>
@@ -5771,13 +5759,13 @@
         <v>53</v>
       </c>
       <c r="E185" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F185" t="s">
         <v>85</v>
       </c>
       <c r="G185" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="I185" s="3"/>
     </row>
@@ -5786,20 +5774,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <dataValidations count="5">
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="Hours are a number above 0 — leave it blank to keep what ships." sqref="I10:I95">
+  <dataValidations count="2">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="Hours are a number above 0 — leave it blank to keep what ships." sqref="I10:I185">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="Hours are a number above 0 — leave it blank to keep what ships." sqref="I100:I185">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="Hours are a number above 0 — leave it blank to keep what ships." sqref="I3:I95">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="textLength" operator="equal" allowBlank="1" showErrorMessage="1" error="HELD — this starter is not seeded yet. Leave it blank." sqref="I96">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="Hours are a number above 0 — leave it blank to keep what ships." sqref="I97:I185">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="Hours are a number above 0 — leave it blank to keep what ships." sqref="I3:I185">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -5819,58 +5798,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>450</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>452</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>454</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>456</v>
+      <c r="B4" s="5" t="s">
+        <v>455</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>457</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>459</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>461</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Catalog review: CI fixes - American spelling in the new rows, the seed test removes the shared rows it inserts on a fresh database, the rename test allows a retired target to be absent; pricing sheets rebuilt (1,793 rows; 0 typed values before); live release plan gains 0140 and § 5d
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pricing/assembly-hours-starter.xlsx
+++ b/pricing/assembly-hours-starter.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="462">
-  <si>
-    <t>STARTER ASSEMBLY HOURS — every starter (183, 15 NEW since the last version — filter the 'New' column). Your top-30 commercial list first, then the top-30 residential, then the rest. Type YELLOW 'MY HOURS' per assembly (one installed). 'Hours now' is what ships today (blank = not set). Leave blank to keep it. Grey = HELD, leave blank. Send the file back to Track A — do NOT edit hours in the app for this.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="461">
+  <si>
+    <t>STARTER ASSEMBLY HOURS — every starter (183, 0 NEW since the last version — filter the 'New' column). Your top-30 commercial list first, then the top-30 residential, then the rest. Type YELLOW 'MY HOURS' per assembly (one installed). 'Hours now' is what ships today (blank = not set). Leave blank to keep it. Grey = HELD, leave blank. Send the file back to Track A — do NOT edit hours in the app for this.</t>
   </si>
   <si>
     <t>#</t>
@@ -824,9 +824,6 @@
     <t>Surface raceway receptacle (block wall)</t>
   </si>
   <si>
-    <t>NEW</t>
-  </si>
-  <si>
     <t>GC5</t>
   </si>
   <si>
@@ -1379,7 +1376,7 @@
     <t>Your top-30 commercial list, then the top-30 residential list (references/top-assemblies-draft.md), then every other starter by category.</t>
   </si>
   <si>
-    <t>15 rows say NEW: starters added since the version this was compared with (ah-previous.xlsx). Filter the 'New' column to see only them.</t>
+    <t>0 rows say NEW: starters added since the version this was compared with (assembly-hours-prev.xlsx). Filter the 'New' column to see only them.</t>
   </si>
   <si>
     <t>HELD</t>
@@ -1416,7 +1413,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1426,11 +1423,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2A8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1446,14 +1438,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3856,23 +3847,20 @@
       <c r="A97">
         <v>95</v>
       </c>
-      <c r="B97" s="4" t="s">
+      <c r="C97" t="s">
+        <v>201</v>
+      </c>
+      <c r="D97" t="s">
+        <v>12</v>
+      </c>
+      <c r="E97" t="s">
         <v>270</v>
-      </c>
-      <c r="C97" t="s">
-        <v>201</v>
-      </c>
-      <c r="D97" t="s">
-        <v>12</v>
-      </c>
-      <c r="E97" t="s">
-        <v>271</v>
       </c>
       <c r="F97" t="s">
         <v>18</v>
       </c>
       <c r="G97" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I97" s="3"/>
     </row>
@@ -3880,9 +3868,6 @@
       <c r="A98">
         <v>96</v>
       </c>
-      <c r="B98" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C98" t="s">
         <v>201</v>
       </c>
@@ -3890,13 +3875,13 @@
         <v>138</v>
       </c>
       <c r="E98" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F98" t="s">
         <v>18</v>
       </c>
       <c r="G98" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I98" s="3"/>
     </row>
@@ -3904,9 +3889,6 @@
       <c r="A99">
         <v>97</v>
       </c>
-      <c r="B99" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C99" t="s">
         <v>201</v>
       </c>
@@ -3914,13 +3896,13 @@
         <v>138</v>
       </c>
       <c r="E99" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F99" t="s">
         <v>18</v>
       </c>
       <c r="G99" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I99" s="3"/>
     </row>
@@ -3928,9 +3910,6 @@
       <c r="A100">
         <v>98</v>
       </c>
-      <c r="B100" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C100" t="s">
         <v>201</v>
       </c>
@@ -3938,13 +3917,13 @@
         <v>138</v>
       </c>
       <c r="E100" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F100" t="s">
         <v>18</v>
       </c>
       <c r="G100" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I100" s="3"/>
     </row>
@@ -3959,13 +3938,13 @@
         <v>12</v>
       </c>
       <c r="E101" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F101" t="s">
         <v>105</v>
       </c>
       <c r="G101" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I101" s="3"/>
     </row>
@@ -3980,13 +3959,13 @@
         <v>12</v>
       </c>
       <c r="E102" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F102" t="s">
         <v>105</v>
       </c>
       <c r="G102" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="I102" s="3"/>
     </row>
@@ -4001,13 +3980,13 @@
         <v>12</v>
       </c>
       <c r="E103" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F103" t="s">
         <v>105</v>
       </c>
       <c r="G103" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I103" s="3"/>
     </row>
@@ -4022,13 +4001,13 @@
         <v>12</v>
       </c>
       <c r="E104" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F104" t="s">
         <v>105</v>
       </c>
       <c r="G104" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="I104" s="3"/>
     </row>
@@ -4043,13 +4022,13 @@
         <v>138</v>
       </c>
       <c r="E105" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F105" t="s">
         <v>105</v>
       </c>
       <c r="G105" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I105" s="3"/>
     </row>
@@ -4064,13 +4043,13 @@
         <v>138</v>
       </c>
       <c r="E106" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F106" t="s">
         <v>105</v>
       </c>
       <c r="G106" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I106" s="3"/>
     </row>
@@ -4085,13 +4064,13 @@
         <v>138</v>
       </c>
       <c r="E107" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F107" t="s">
         <v>105</v>
       </c>
       <c r="G107" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I107" s="3"/>
     </row>
@@ -4106,13 +4085,13 @@
         <v>12</v>
       </c>
       <c r="E108" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F108" t="s">
         <v>105</v>
       </c>
       <c r="G108" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I108" s="3"/>
     </row>
@@ -4127,13 +4106,13 @@
         <v>12</v>
       </c>
       <c r="E109" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F109" t="s">
         <v>105</v>
       </c>
       <c r="G109" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I109" s="3"/>
     </row>
@@ -4148,13 +4127,13 @@
         <v>12</v>
       </c>
       <c r="E110" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F110" t="s">
         <v>105</v>
       </c>
       <c r="G110" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I110" s="3"/>
     </row>
@@ -4169,13 +4148,13 @@
         <v>12</v>
       </c>
       <c r="E111" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F111" t="s">
         <v>105</v>
       </c>
       <c r="G111" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I111" s="3"/>
     </row>
@@ -4190,13 +4169,13 @@
         <v>12</v>
       </c>
       <c r="E112" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F112" t="s">
         <v>105</v>
       </c>
       <c r="G112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I112" s="3"/>
     </row>
@@ -4211,13 +4190,13 @@
         <v>12</v>
       </c>
       <c r="E113" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F113" t="s">
         <v>105</v>
       </c>
       <c r="G113" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I113" s="3"/>
     </row>
@@ -4232,13 +4211,13 @@
         <v>12</v>
       </c>
       <c r="E114" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F114" t="s">
         <v>105</v>
       </c>
       <c r="G114" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I114" s="3"/>
     </row>
@@ -4253,13 +4232,13 @@
         <v>138</v>
       </c>
       <c r="E115" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F115" t="s">
         <v>105</v>
       </c>
       <c r="G115" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I115" s="3"/>
     </row>
@@ -4274,13 +4253,13 @@
         <v>53</v>
       </c>
       <c r="E116" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F116" t="s">
         <v>105</v>
       </c>
       <c r="G116" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I116" s="3"/>
     </row>
@@ -4295,13 +4274,13 @@
         <v>138</v>
       </c>
       <c r="E117" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F117" t="s">
         <v>105</v>
       </c>
       <c r="G117" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I117" s="3"/>
     </row>
@@ -4316,13 +4295,13 @@
         <v>138</v>
       </c>
       <c r="E118" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F118" t="s">
         <v>105</v>
       </c>
       <c r="G118" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="I118" s="3"/>
     </row>
@@ -4337,13 +4316,13 @@
         <v>138</v>
       </c>
       <c r="E119" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F119" t="s">
         <v>105</v>
       </c>
       <c r="G119" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="I119" s="3"/>
     </row>
@@ -4358,13 +4337,13 @@
         <v>138</v>
       </c>
       <c r="E120" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F120" t="s">
         <v>105</v>
       </c>
       <c r="G120" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I120" s="3"/>
     </row>
@@ -4379,13 +4358,13 @@
         <v>138</v>
       </c>
       <c r="E121" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F121" t="s">
         <v>105</v>
       </c>
       <c r="G121" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I121" s="3"/>
     </row>
@@ -4400,13 +4379,13 @@
         <v>138</v>
       </c>
       <c r="E122" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F122" t="s">
         <v>105</v>
       </c>
       <c r="G122" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="I122" s="3"/>
     </row>
@@ -4421,13 +4400,13 @@
         <v>138</v>
       </c>
       <c r="E123" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F123" t="s">
         <v>105</v>
       </c>
       <c r="G123" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="I123" s="3"/>
     </row>
@@ -4442,13 +4421,13 @@
         <v>138</v>
       </c>
       <c r="E124" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F124" t="s">
         <v>105</v>
       </c>
       <c r="G124" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="I124" s="3"/>
     </row>
@@ -4463,13 +4442,13 @@
         <v>12</v>
       </c>
       <c r="E125" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F125" t="s">
         <v>41</v>
       </c>
       <c r="G125" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="I125" s="3"/>
     </row>
@@ -4484,13 +4463,13 @@
         <v>53</v>
       </c>
       <c r="E126" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F126" t="s">
         <v>41</v>
       </c>
       <c r="G126" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I126" s="3"/>
     </row>
@@ -4505,13 +4484,13 @@
         <v>12</v>
       </c>
       <c r="E127" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F127" t="s">
         <v>41</v>
       </c>
       <c r="G127" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="I127" s="3"/>
     </row>
@@ -4526,13 +4505,13 @@
         <v>53</v>
       </c>
       <c r="E128" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F128" t="s">
         <v>41</v>
       </c>
       <c r="G128" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="I128" s="3"/>
     </row>
@@ -4547,13 +4526,13 @@
         <v>12</v>
       </c>
       <c r="E129" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F129" t="s">
         <v>41</v>
       </c>
       <c r="G129" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="I129" s="3"/>
     </row>
@@ -4568,13 +4547,13 @@
         <v>138</v>
       </c>
       <c r="E130" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F130" t="s">
         <v>41</v>
       </c>
       <c r="G130" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I130" s="3"/>
     </row>
@@ -4589,13 +4568,13 @@
         <v>53</v>
       </c>
       <c r="E131" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F131" t="s">
         <v>41</v>
       </c>
       <c r="G131" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="I131" s="3"/>
     </row>
@@ -4610,13 +4589,13 @@
         <v>53</v>
       </c>
       <c r="E132" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F132" t="s">
         <v>41</v>
       </c>
       <c r="G132" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="I132" s="3"/>
     </row>
@@ -4631,13 +4610,13 @@
         <v>12</v>
       </c>
       <c r="E133" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F133" t="s">
         <v>14</v>
       </c>
       <c r="G133" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="I133" s="3"/>
     </row>
@@ -4645,9 +4624,6 @@
       <c r="A134">
         <v>132</v>
       </c>
-      <c r="B134" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C134" t="s">
         <v>201</v>
       </c>
@@ -4655,13 +4631,13 @@
         <v>12</v>
       </c>
       <c r="E134" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F134" t="s">
         <v>14</v>
       </c>
       <c r="G134" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="I134" s="3"/>
     </row>
@@ -4669,9 +4645,6 @@
       <c r="A135">
         <v>133</v>
       </c>
-      <c r="B135" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C135" t="s">
         <v>201</v>
       </c>
@@ -4679,13 +4652,13 @@
         <v>12</v>
       </c>
       <c r="E135" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F135" t="s">
         <v>14</v>
       </c>
       <c r="G135" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="I135" s="3"/>
     </row>
@@ -4693,9 +4666,6 @@
       <c r="A136">
         <v>134</v>
       </c>
-      <c r="B136" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C136" t="s">
         <v>201</v>
       </c>
@@ -4703,13 +4673,13 @@
         <v>12</v>
       </c>
       <c r="E136" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F136" t="s">
         <v>14</v>
       </c>
       <c r="G136" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="I136" s="3"/>
     </row>
@@ -4724,13 +4694,13 @@
         <v>138</v>
       </c>
       <c r="E137" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F137" t="s">
         <v>14</v>
       </c>
       <c r="G137" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I137" s="3"/>
     </row>
@@ -4745,13 +4715,13 @@
         <v>53</v>
       </c>
       <c r="E138" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F138" t="s">
         <v>14</v>
       </c>
       <c r="G138" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="I138" s="3"/>
     </row>
@@ -4766,13 +4736,13 @@
         <v>53</v>
       </c>
       <c r="E139" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="F139" t="s">
         <v>14</v>
       </c>
       <c r="G139" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I139" s="3"/>
     </row>
@@ -4787,13 +4757,13 @@
         <v>53</v>
       </c>
       <c r="E140" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F140" t="s">
         <v>14</v>
       </c>
       <c r="G140" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I140" s="3"/>
     </row>
@@ -4808,13 +4778,13 @@
         <v>138</v>
       </c>
       <c r="E141" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F141" t="s">
         <v>14</v>
       </c>
       <c r="G141" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I141" s="3"/>
     </row>
@@ -4829,13 +4799,13 @@
         <v>138</v>
       </c>
       <c r="E142" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F142" t="s">
         <v>14</v>
       </c>
       <c r="G142" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I142" s="3"/>
     </row>
@@ -4850,13 +4820,13 @@
         <v>138</v>
       </c>
       <c r="E143" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F143" t="s">
         <v>14</v>
       </c>
       <c r="G143" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I143" s="3"/>
     </row>
@@ -4871,13 +4841,13 @@
         <v>138</v>
       </c>
       <c r="E144" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F144" t="s">
         <v>14</v>
       </c>
       <c r="G144" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I144" s="3"/>
     </row>
@@ -4892,13 +4862,13 @@
         <v>53</v>
       </c>
       <c r="E145" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F145" t="s">
         <v>14</v>
       </c>
       <c r="G145" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="I145" s="3"/>
     </row>
@@ -4913,13 +4883,13 @@
         <v>138</v>
       </c>
       <c r="E146" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F146" t="s">
         <v>14</v>
       </c>
       <c r="G146" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="I146" s="3"/>
     </row>
@@ -4934,13 +4904,13 @@
         <v>138</v>
       </c>
       <c r="E147" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F147" t="s">
         <v>14</v>
       </c>
       <c r="G147" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I147" s="3"/>
     </row>
@@ -4955,13 +4925,13 @@
         <v>12</v>
       </c>
       <c r="E148" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F148" t="s">
         <v>14</v>
       </c>
       <c r="G148" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="I148" s="3"/>
     </row>
@@ -4976,13 +4946,13 @@
         <v>12</v>
       </c>
       <c r="E149" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F149" t="s">
         <v>14</v>
       </c>
       <c r="G149" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="I149" s="3"/>
     </row>
@@ -4997,13 +4967,13 @@
         <v>12</v>
       </c>
       <c r="E150" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F150" t="s">
         <v>14</v>
       </c>
       <c r="G150" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="I150" s="3"/>
     </row>
@@ -5018,13 +4988,13 @@
         <v>12</v>
       </c>
       <c r="E151" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F151" t="s">
         <v>14</v>
       </c>
       <c r="G151" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="I151" s="3"/>
     </row>
@@ -5039,13 +5009,13 @@
         <v>12</v>
       </c>
       <c r="E152" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F152" t="s">
         <v>14</v>
       </c>
       <c r="G152" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I152" s="3"/>
     </row>
@@ -5053,9 +5023,6 @@
       <c r="A153">
         <v>151</v>
       </c>
-      <c r="B153" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C153" t="s">
         <v>201</v>
       </c>
@@ -5063,13 +5030,13 @@
         <v>53</v>
       </c>
       <c r="E153" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F153" t="s">
         <v>14</v>
       </c>
       <c r="G153" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="I153" s="3"/>
     </row>
@@ -5077,9 +5044,6 @@
       <c r="A154">
         <v>152</v>
       </c>
-      <c r="B154" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C154" t="s">
         <v>201</v>
       </c>
@@ -5087,13 +5051,13 @@
         <v>53</v>
       </c>
       <c r="E154" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F154" t="s">
         <v>14</v>
       </c>
       <c r="G154" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="I154" s="3"/>
     </row>
@@ -5101,9 +5065,6 @@
       <c r="A155">
         <v>153</v>
       </c>
-      <c r="B155" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C155" t="s">
         <v>201</v>
       </c>
@@ -5111,13 +5072,13 @@
         <v>53</v>
       </c>
       <c r="E155" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F155" t="s">
         <v>14</v>
       </c>
       <c r="G155" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="I155" s="3"/>
     </row>
@@ -5132,13 +5093,13 @@
         <v>12</v>
       </c>
       <c r="E156" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F156" t="s">
         <v>89</v>
       </c>
       <c r="G156" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="I156" s="3"/>
     </row>
@@ -5153,13 +5114,13 @@
         <v>12</v>
       </c>
       <c r="E157" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F157" t="s">
         <v>89</v>
       </c>
       <c r="G157" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="I157" s="3"/>
     </row>
@@ -5174,13 +5135,13 @@
         <v>12</v>
       </c>
       <c r="E158" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F158" t="s">
         <v>89</v>
       </c>
       <c r="G158" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I158" s="3"/>
     </row>
@@ -5195,13 +5156,13 @@
         <v>12</v>
       </c>
       <c r="E159" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F159" t="s">
         <v>89</v>
       </c>
       <c r="G159" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I159" s="3"/>
     </row>
@@ -5216,13 +5177,13 @@
         <v>138</v>
       </c>
       <c r="E160" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F160" t="s">
         <v>89</v>
       </c>
       <c r="G160" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="I160" s="3"/>
     </row>
@@ -5237,13 +5198,13 @@
         <v>138</v>
       </c>
       <c r="E161" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F161" t="s">
         <v>89</v>
       </c>
       <c r="G161" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="I161" s="3"/>
     </row>
@@ -5258,13 +5219,13 @@
         <v>53</v>
       </c>
       <c r="E162" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F162" t="s">
         <v>89</v>
       </c>
       <c r="G162" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="I162" s="3"/>
     </row>
@@ -5279,13 +5240,13 @@
         <v>138</v>
       </c>
       <c r="E163" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F163" t="s">
         <v>89</v>
       </c>
       <c r="G163" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="I163" s="3"/>
     </row>
@@ -5300,13 +5261,13 @@
         <v>12</v>
       </c>
       <c r="E164" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F164" t="s">
         <v>89</v>
       </c>
       <c r="G164" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I164" s="3"/>
     </row>
@@ -5321,13 +5282,13 @@
         <v>138</v>
       </c>
       <c r="E165" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F165" t="s">
         <v>89</v>
       </c>
       <c r="G165" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="I165" s="3"/>
     </row>
@@ -5342,13 +5303,13 @@
         <v>138</v>
       </c>
       <c r="E166" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F166" t="s">
         <v>89</v>
       </c>
       <c r="G166" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="I166" s="3"/>
     </row>
@@ -5356,9 +5317,6 @@
       <c r="A167">
         <v>165</v>
       </c>
-      <c r="B167" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C167" t="s">
         <v>201</v>
       </c>
@@ -5366,13 +5324,13 @@
         <v>12</v>
       </c>
       <c r="E167" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F167" t="s">
         <v>85</v>
       </c>
       <c r="G167" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="I167" s="3"/>
     </row>
@@ -5380,9 +5338,6 @@
       <c r="A168">
         <v>166</v>
       </c>
-      <c r="B168" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C168" t="s">
         <v>201</v>
       </c>
@@ -5390,13 +5345,13 @@
         <v>138</v>
       </c>
       <c r="E168" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F168" t="s">
         <v>85</v>
       </c>
       <c r="G168" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="I168" s="3"/>
     </row>
@@ -5404,9 +5359,6 @@
       <c r="A169">
         <v>167</v>
       </c>
-      <c r="B169" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C169" t="s">
         <v>201</v>
       </c>
@@ -5414,13 +5366,13 @@
         <v>138</v>
       </c>
       <c r="E169" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F169" t="s">
         <v>85</v>
       </c>
       <c r="G169" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="I169" s="3"/>
     </row>
@@ -5428,9 +5380,6 @@
       <c r="A170">
         <v>168</v>
       </c>
-      <c r="B170" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C170" t="s">
         <v>201</v>
       </c>
@@ -5438,13 +5387,13 @@
         <v>138</v>
       </c>
       <c r="E170" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="F170" t="s">
         <v>85</v>
       </c>
       <c r="G170" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I170" s="3"/>
     </row>
@@ -5452,9 +5401,6 @@
       <c r="A171">
         <v>169</v>
       </c>
-      <c r="B171" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="C171" t="s">
         <v>201</v>
       </c>
@@ -5462,13 +5408,13 @@
         <v>138</v>
       </c>
       <c r="E171" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F171" t="s">
         <v>85</v>
       </c>
       <c r="G171" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="I171" s="3"/>
     </row>
@@ -5483,13 +5429,13 @@
         <v>53</v>
       </c>
       <c r="E172" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="F172" t="s">
         <v>85</v>
       </c>
       <c r="G172" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="H172">
         <v>8</v>
@@ -5507,13 +5453,13 @@
         <v>53</v>
       </c>
       <c r="E173" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="F173" t="s">
         <v>85</v>
       </c>
       <c r="G173" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="I173" s="3"/>
     </row>
@@ -5528,13 +5474,13 @@
         <v>138</v>
       </c>
       <c r="E174" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F174" t="s">
         <v>85</v>
       </c>
       <c r="G174" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I174" s="3"/>
     </row>
@@ -5549,13 +5495,13 @@
         <v>53</v>
       </c>
       <c r="E175" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="F175" t="s">
         <v>85</v>
       </c>
       <c r="G175" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I175" s="3"/>
     </row>
@@ -5570,13 +5516,13 @@
         <v>53</v>
       </c>
       <c r="E176" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="F176" t="s">
         <v>85</v>
       </c>
       <c r="G176" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="I176" s="3"/>
     </row>
@@ -5591,13 +5537,13 @@
         <v>138</v>
       </c>
       <c r="E177" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F177" t="s">
         <v>85</v>
       </c>
       <c r="G177" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I177" s="3"/>
     </row>
@@ -5612,13 +5558,13 @@
         <v>53</v>
       </c>
       <c r="E178" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="F178" t="s">
         <v>85</v>
       </c>
       <c r="G178" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="I178" s="3"/>
     </row>
@@ -5633,13 +5579,13 @@
         <v>12</v>
       </c>
       <c r="E179" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F179" t="s">
         <v>85</v>
       </c>
       <c r="G179" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="I179" s="3"/>
     </row>
@@ -5654,13 +5600,13 @@
         <v>12</v>
       </c>
       <c r="E180" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="F180" t="s">
         <v>85</v>
       </c>
       <c r="G180" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="I180" s="3"/>
     </row>
@@ -5675,13 +5621,13 @@
         <v>12</v>
       </c>
       <c r="E181" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F181" t="s">
         <v>85</v>
       </c>
       <c r="G181" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="I181" s="3"/>
     </row>
@@ -5696,13 +5642,13 @@
         <v>12</v>
       </c>
       <c r="E182" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F182" t="s">
         <v>85</v>
       </c>
       <c r="G182" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I182" s="3"/>
     </row>
@@ -5717,13 +5663,13 @@
         <v>53</v>
       </c>
       <c r="E183" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F183" t="s">
         <v>85</v>
       </c>
       <c r="G183" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="I183" s="3"/>
     </row>
@@ -5738,13 +5684,13 @@
         <v>12</v>
       </c>
       <c r="E184" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F184" t="s">
         <v>85</v>
       </c>
       <c r="G184" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="I184" s="3"/>
     </row>
@@ -5759,13 +5705,13 @@
         <v>53</v>
       </c>
       <c r="E185" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="F185" t="s">
         <v>85</v>
       </c>
       <c r="G185" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="I185" s="3"/>
     </row>
@@ -5798,58 +5744,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>449</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>451</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>453</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>455</v>
+      <c r="B4" s="4" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>456</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>458</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>460</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>